<commit_message>
Limit demo package to four agreed business tasks
</commit_message>
<xml_diff>
--- a/DEMO_ACCEPTANCE.xlsx
+++ b/DEMO_ACCEPTANCE.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验收清单" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'验收清单'!$A$1:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'验收清单'!$A$1:$F$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -889,40 +889,9 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>指标</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>业务ROI</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>记录基线与试点数据后比较</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>待测量</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>尚无生产样本</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>不填写虚构提升百分比</t>
-        </is>
-      </c>
-    </row>
+    <row r="15" ht="42" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:F15"/>
+  <autoFilter ref="A1:F14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>